<commit_message>
restructure specification incl. appendices, auto-inject ref data
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pva/work/github.com/doclang-project/doclang-standard/reference/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7A814EF-C50D-004B-948D-8458FD1A3094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E5F33BA-4BB4-1B4A-9E0B-B0223A046B88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="2" xr2:uid="{53E75A16-C0D6-3446-9F63-761042DEAA14}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="1" xr2:uid="{53E75A16-C0D6-3446-9F63-761042DEAA14}"/>
   </bookViews>
   <sheets>
     <sheet name="categories" sheetId="4" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="180">
   <si>
     <t>{"read_only", "fillable"}</t>
   </si>
@@ -66,9 +66,6 @@
   </si>
   <si>
     <t>Element</t>
-  </si>
-  <si>
-    <t>Includes doc-level metadata.</t>
   </si>
   <si>
     <t>Exists exactly once, as root element.</t>
@@ -424,9 +421,6 @@
     <t>special</t>
   </si>
   <si>
-    <t>grouping</t>
-  </si>
-  <si>
     <t>component head</t>
   </si>
   <si>
@@ -487,9 +481,6 @@
     <t>Formatting elements modify the styling and presentation within semantic or other formatting elements.</t>
   </si>
   <si>
-    <t>Structural elements define boundaries within tabular content (`&lt;otsl&gt;`).</t>
-  </si>
-  <si>
     <t>This category comprises elements with specialized document-level function.</t>
   </si>
   <si>
@@ -505,18 +496,10 @@
     <t>[Content] Raw text</t>
   </si>
   <si>
-    <t>Grouping elements enable the encapsulation of semantic elements or other grouping elements. Any grouping element may optionally begin with a [component head](#component-head-elements).</t>
-  </si>
-  <si>
     <t>Element Allowed Context</t>
   </si>
   <si>
     <t>Element Description</t>
-  </si>
-  <si>
-    <t>The component head is a sequence comprising the following elements in this order, whereby all elements are optional:&lt;br /&gt;&lt;ul&gt;&lt;li&gt;`&lt;thread&gt;`&lt;/li&gt;&lt;li&gt;`&lt;h_thread&gt;`&lt;/li&gt;&lt;li&gt;`&lt;meta&gt;`&lt;/li&gt;&lt;li&gt;sequence of 2*N `&lt;location&gt;`s (N&gt;1)&lt;/li&gt;&lt;li&gt;sequence of `&lt;timestamp&gt;`s&lt;/li&gt;&lt;li&gt;`&lt;layer&gt;`&lt;/li&gt;&lt;/ul&gt;
-A component head can only appear as the leading content of a semantic or grouping element, or also of `&lt;otsl&gt;` in the context of "implicit `&lt;text&gt;`s".&lt;br/&gt;
-The various component head elements are further specified in the following subsections.</t>
   </si>
   <si>
     <t>Any context that allows raw text content.</t>
@@ -593,6 +576,17 @@
   </si>
   <si>
     <t>The DocLang specification version the document is supposed to validate against, in "MAJOR.MINOR" format, i.e. first two positions of Semantic Verisoning.</t>
+  </si>
+  <si>
+    <t>The component head is a sequence comprising the following elements in this order, whereby all elements are optional:&lt;br /&gt;&lt;ul&gt;&lt;li&gt;`&lt;thread&gt;`&lt;/li&gt;&lt;li&gt;`&lt;h_thread&gt;`&lt;/li&gt;&lt;li&gt;`&lt;meta&gt;`&lt;/li&gt;&lt;li&gt;sequence of 2*N `&lt;location&gt;`s (N&gt;1)&lt;/li&gt;&lt;li&gt;sequence of `&lt;timestamp&gt;`s&lt;/li&gt;&lt;li&gt;`&lt;layer&gt;`&lt;/li&gt;&lt;/ul&gt;
+A component head can only appear as the leading content of a semantic element.
+The various component head elements are further specified in the following subsections.</t>
+  </si>
+  <si>
+    <t>Structural elements define boundaries within explicitly structured components like tables and lists.</t>
+  </si>
+  <si>
+    <t>Includes doc-level metadata. Also discussed in Appendix B.</t>
   </si>
 </sst>
 </file>
@@ -1000,7 +994,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AD32FCC-87C5-AA40-8339-205A5A3F17B2}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
@@ -1009,74 +1003,66 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" t="s">
         <v>121</v>
-      </c>
-      <c r="B1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="85" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="85" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="B4" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="102" x14ac:dyDescent="0.2">
-      <c r="A5" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>156</v>
+      <c r="B5" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B7" t="s">
-        <v>146</v>
+        <v>178</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="B8" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="B9" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -1106,62 +1092,62 @@
         <v>7</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="D2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G2" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H2" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="34" x14ac:dyDescent="0.2">
+      <c r="A3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F2" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G2" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H2" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="17" x14ac:dyDescent="0.2">
-      <c r="A3" s="7" t="s">
-        <v>10</v>
-      </c>
       <c r="B3" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>8</v>
+        <v>179</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E3" s="6" t="b">
         <v>1</v>
@@ -1178,16 +1164,16 @@
     </row>
     <row r="4" spans="1:8" ht="136" x14ac:dyDescent="0.2">
       <c r="A4" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E4" s="6" t="b">
         <v>0</v>
@@ -1204,16 +1190,16 @@
     </row>
     <row r="5" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E5" s="6" t="b">
         <v>1</v>
@@ -1230,14 +1216,14 @@
     </row>
     <row r="6" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E6" s="6" t="b">
         <v>1</v>
@@ -1254,14 +1240,14 @@
     </row>
     <row r="7" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E7" s="6" t="b">
         <v>1</v>
@@ -1278,14 +1264,14 @@
     </row>
     <row r="8" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E8" s="6" t="b">
         <v>1</v>
@@ -1302,14 +1288,14 @@
     </row>
     <row r="9" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E9" s="6" t="b">
         <v>1</v>
@@ -1326,14 +1312,14 @@
     </row>
     <row r="10" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E10" s="6" t="b">
         <v>1</v>
@@ -1350,16 +1336,16 @@
     </row>
     <row r="11" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E11" s="6" t="b">
         <v>1</v>
@@ -1376,16 +1362,16 @@
     </row>
     <row r="12" spans="1:8" ht="51" x14ac:dyDescent="0.2">
       <c r="A12" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E12" s="6" t="b">
         <v>1</v>
@@ -1402,16 +1388,16 @@
     </row>
     <row r="13" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E13" s="6" t="b">
         <v>1</v>
@@ -1428,14 +1414,14 @@
     </row>
     <row r="14" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A14" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C14" s="5"/>
       <c r="D14" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E14" s="6" t="b">
         <v>1</v>
@@ -1452,14 +1438,14 @@
     </row>
     <row r="15" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A15" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E15" s="6" t="b">
         <v>1</v>
@@ -1476,14 +1462,14 @@
     </row>
     <row r="16" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E16" s="6" t="b">
         <v>1</v>
@@ -1500,14 +1486,14 @@
     </row>
     <row r="17" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C17" s="5"/>
       <c r="D17" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E17" s="6" t="b">
         <v>1</v>
@@ -1524,16 +1510,16 @@
     </row>
     <row r="18" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E18" s="6" t="b">
         <v>1</v>
@@ -1550,14 +1536,14 @@
     </row>
     <row r="19" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C19" s="5"/>
       <c r="D19" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E19" s="6" t="b">
         <v>1</v>
@@ -1574,16 +1560,16 @@
     </row>
     <row r="20" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A20" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E20" s="6" t="b">
         <v>1</v>
@@ -1600,16 +1586,16 @@
     </row>
     <row r="21" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E21" s="6" t="b">
         <v>1</v>
@@ -1626,16 +1612,16 @@
     </row>
     <row r="22" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E22" s="6" t="b">
         <v>1</v>
@@ -1652,16 +1638,16 @@
     </row>
     <row r="23" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E23" s="6" t="b">
         <v>1</v>
@@ -1678,16 +1664,16 @@
     </row>
     <row r="24" spans="1:8" ht="153" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="E24" s="6" t="b">
         <v>0</v>
@@ -1704,16 +1690,16 @@
     </row>
     <row r="25" spans="1:8" ht="68" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="E25" s="6" t="b">
         <v>0</v>
@@ -1730,16 +1716,16 @@
     </row>
     <row r="26" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="E26" s="6" t="b">
         <v>1</v>
@@ -1756,16 +1742,16 @@
     </row>
     <row r="27" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="E27" s="6" t="b">
         <v>1</v>
@@ -1782,16 +1768,16 @@
     </row>
     <row r="28" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A28" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="E28" s="6" t="b">
         <v>0</v>
@@ -1808,16 +1794,16 @@
     </row>
     <row r="29" spans="1:8" ht="85" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="E29" s="6" t="b">
         <v>1</v>
@@ -1834,14 +1820,14 @@
     </row>
     <row r="30" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A30" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C30" s="5"/>
       <c r="D30" s="6" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="E30" s="6" t="b">
         <v>0</v>
@@ -1858,14 +1844,14 @@
     </row>
     <row r="31" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="6" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="E31" s="6" t="b">
         <v>0</v>
@@ -1882,14 +1868,14 @@
     </row>
     <row r="32" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A32" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="6" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="E32" s="6" t="b">
         <v>0</v>
@@ -1906,14 +1892,14 @@
     </row>
     <row r="33" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A33" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C33" s="5"/>
       <c r="D33" s="6" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="E33" s="6" t="b">
         <v>0</v>
@@ -1930,14 +1916,14 @@
     </row>
     <row r="34" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A34" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C34" s="5"/>
       <c r="D34" s="6" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="E34" s="6" t="b">
         <v>0</v>
@@ -1954,14 +1940,14 @@
     </row>
     <row r="35" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A35" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C35" s="5"/>
       <c r="D35" s="5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E35" s="6" t="b">
         <v>1</v>
@@ -1978,14 +1964,14 @@
     </row>
     <row r="36" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A36" s="7" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C36" s="5"/>
       <c r="D36" s="5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E36" s="6" t="b">
         <v>1</v>
@@ -2002,16 +1988,16 @@
     </row>
     <row r="37" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A37" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E37" s="6" t="b">
         <v>1</v>
@@ -2028,14 +2014,14 @@
     </row>
     <row r="38" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C38" s="5"/>
       <c r="D38" s="5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="E38" s="6" t="b">
         <v>0</v>
@@ -2052,14 +2038,14 @@
     </row>
     <row r="39" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C39" s="5"/>
       <c r="D39" s="5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="E39" s="6" t="b">
         <v>1</v>
@@ -2076,14 +2062,14 @@
     </row>
     <row r="40" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A40" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C40" s="5"/>
       <c r="D40" s="5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="E40" s="6" t="b">
         <v>1</v>
@@ -2100,14 +2086,14 @@
     </row>
     <row r="41" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A41" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C41" s="5"/>
       <c r="D41" s="5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="E41" s="6" t="b">
         <v>1</v>
@@ -2124,14 +2110,14 @@
     </row>
     <row r="42" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A42" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C42" s="5"/>
       <c r="D42" s="5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="E42" s="6" t="b">
         <v>1</v>
@@ -2148,14 +2134,14 @@
     </row>
     <row r="43" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A43" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C43" s="5"/>
       <c r="D43" s="5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="E43" s="6" t="b">
         <v>1</v>
@@ -2172,14 +2158,14 @@
     </row>
     <row r="44" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A44" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C44" s="5"/>
       <c r="D44" s="5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="E44" s="6" t="b">
         <v>1</v>
@@ -2196,14 +2182,14 @@
     </row>
     <row r="45" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A45" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C45" s="5"/>
       <c r="D45" s="5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="E45" s="6" t="b">
         <v>1</v>
@@ -2220,14 +2206,14 @@
     </row>
     <row r="46" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A46" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C46" s="5"/>
       <c r="D46" s="5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="E46" s="6" t="b">
         <v>1</v>
@@ -2244,16 +2230,16 @@
     </row>
     <row r="47" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="E47" s="6" t="b">
         <v>1</v>
@@ -2270,16 +2256,16 @@
     </row>
     <row r="48" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A48" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="E48" s="6" t="b">
         <v>1</v>
@@ -2296,14 +2282,14 @@
     </row>
     <row r="49" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A49" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C49" s="5"/>
       <c r="D49" s="5" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="E49" s="6" t="b">
         <v>0</v>
@@ -2320,14 +2306,14 @@
     </row>
     <row r="50" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A50" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C50" s="5"/>
       <c r="D50" s="5" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="E50" s="6" t="b">
         <v>0</v>
@@ -2344,14 +2330,14 @@
     </row>
     <row r="51" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A51" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C51" s="5"/>
       <c r="D51" s="5" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="E51" s="6" t="b">
         <v>0</v>
@@ -2368,14 +2354,14 @@
     </row>
     <row r="52" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C52" s="5"/>
       <c r="D52" s="5" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="E52" s="6" t="b">
         <v>0</v>
@@ -2392,14 +2378,14 @@
     </row>
     <row r="53" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A53" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C53" s="5"/>
       <c r="D53" s="5" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="E53" s="6" t="b">
         <v>0</v>
@@ -2416,14 +2402,14 @@
     </row>
     <row r="54" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A54" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C54" s="5"/>
       <c r="D54" s="5" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="E54" s="6" t="b">
         <v>0</v>
@@ -2440,14 +2426,14 @@
     </row>
     <row r="55" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A55" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C55" s="5"/>
       <c r="D55" s="5" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="E55" s="6" t="b">
         <v>0</v>
@@ -2464,14 +2450,14 @@
     </row>
     <row r="56" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A56" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C56" s="5"/>
       <c r="D56" s="5" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="E56" s="6" t="b">
         <v>0</v>
@@ -2488,14 +2474,14 @@
     </row>
     <row r="57" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A57" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C57" s="5"/>
       <c r="D57" s="5" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="E57" s="6" t="b">
         <v>0</v>
@@ -2512,14 +2498,14 @@
     </row>
     <row r="58" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A58" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C58" s="5"/>
       <c r="D58" s="5" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="E58" s="6" t="b">
         <v>0</v>
@@ -2536,16 +2522,16 @@
     </row>
     <row r="59" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A59" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E59" s="6" t="b">
         <v>1</v>
@@ -2557,15 +2543,15 @@
         <v>0</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
     </row>
     <row r="60" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A60" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C60" s="6" t="s">
         <v>5</v>
@@ -2588,10 +2574,10 @@
     </row>
     <row r="61" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A61" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C61" s="6" t="s">
         <v>5</v>
@@ -2614,10 +2600,10 @@
     </row>
     <row r="62" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A62" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>5</v>
@@ -2640,10 +2626,10 @@
     </row>
     <row r="63" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A63" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C63" s="6" t="s">
         <v>5</v>
@@ -2666,10 +2652,10 @@
     </row>
     <row r="64" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A64" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C64" s="6" t="s">
         <v>5</v>
@@ -2692,10 +2678,10 @@
     </row>
     <row r="65" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A65" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C65" s="6" t="s">
         <v>5</v>
@@ -2718,10 +2704,10 @@
     </row>
     <row r="66" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A66" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C66" s="6" t="s">
         <v>5</v>
@@ -2744,10 +2730,10 @@
     </row>
     <row r="67" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A67" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C67" s="6" t="s">
         <v>5</v>
@@ -2770,10 +2756,10 @@
     </row>
     <row r="68" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A68" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C68" s="6" t="s">
         <v>5</v>
@@ -2796,10 +2782,10 @@
     </row>
     <row r="69" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A69" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C69" s="6" t="s">
         <v>5</v>
@@ -2822,10 +2808,10 @@
     </row>
     <row r="70" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A70" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C70" s="6" t="s">
         <v>5</v>
@@ -2848,10 +2834,10 @@
     </row>
     <row r="71" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A71" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C71" s="6" t="s">
         <v>5</v>
@@ -2874,10 +2860,10 @@
     </row>
     <row r="72" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A72" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C72" s="6" t="s">
         <v>5</v>
@@ -2900,10 +2886,10 @@
     </row>
     <row r="73" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A73" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C73" s="6" t="s">
         <v>5</v>
@@ -2926,10 +2912,10 @@
     </row>
     <row r="74" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A74" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C74" s="6" t="s">
         <v>5</v>
@@ -2952,10 +2938,10 @@
     </row>
     <row r="75" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A75" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C75" s="6" t="s">
         <v>5</v>
@@ -2978,10 +2964,10 @@
     </row>
     <row r="76" spans="1:8" ht="17" x14ac:dyDescent="0.2">
       <c r="A76" s="7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C76" s="6" t="s">
         <v>5</v>
@@ -3036,145 +3022,145 @@
         <v>7</v>
       </c>
       <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
-        <v>18</v>
-      </c>
       <c r="D1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E1" t="s">
         <v>112</v>
-      </c>
-      <c r="E1" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C2" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="D2" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="E2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C3" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="D3" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="E3" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C4" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D4" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D6" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C7" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D7" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C8" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C9" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D9" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C10" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D10" t="s">
         <v>4</v>
@@ -3182,13 +3168,13 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C11" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D11" t="s">
         <v>0</v>
@@ -3196,13 +3182,13 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C12" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D12" t="s">
         <v>3</v>
@@ -3210,13 +3196,13 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B13" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C13" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D13" t="s">
         <v>1</v>
@@ -3224,27 +3210,27 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C14" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C15" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D15" t="s">
         <v>2</v>
@@ -3252,33 +3238,33 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B16" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C16" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D16" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E16" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B17" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C17" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D17" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refine `<picture>` subclassing, update examples (#80)
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="attributes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'attributes'!$A$1:$E$12</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -601,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J82"/>
+  <dimension ref="A1:J81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20" defaultRowHeight="16"/>
   <cols>
     <col width="27.1640625" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -610,8 +610,8 @@
     <col width="36.5" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="20"/>
-    <col width="20" customWidth="1" style="1" min="21" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="21"/>
+    <col width="20" customWidth="1" style="1" min="22" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Can contain a `&lt;src&gt;` for image bytes or reference. Additionally, the element body may begin with a `&lt;table&gt;` in case of `&lt;picture class="chart"&gt;` or with a `&lt;smiles&gt;` in case of `&lt;picture class="chemistry"&gt;`.</t>
+          <t>Can contain a `&lt;src&gt;` for image bytes or reference. Additionally, the element body may begin with a `&lt;table&gt;` in case of `&lt;picture class="chart"&gt;`.</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -2184,22 +2184,18 @@
     <row r="44" ht="17" customHeight="1">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>[04] payload</t>
+          <t>[05] formatting</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>`&lt;smiles&gt;`</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>The SMILES representation of a molecule.</t>
-        </is>
-      </c>
+          <t>`&lt;bold&gt;`</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="n"/>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Can only be the first element of the element body of `&lt;picture class="chemistry"&gt;`.</t>
+          <t>Any context that allows raw text content.</t>
         </is>
       </c>
       <c r="E44" s="6" t="b">
@@ -2208,7 +2204,7 @@
       <c r="F44" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G44" s="1" t="b">
+      <c r="G44" s="6" t="b">
         <v>1</v>
       </c>
       <c r="H44" s="1" t="b">
@@ -2223,7 +2219,7 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>`&lt;bold&gt;`</t>
+          <t>`&lt;italic&gt;`</t>
         </is>
       </c>
       <c r="C45" s="5" t="n"/>
@@ -2253,7 +2249,7 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>`&lt;italic&gt;`</t>
+          <t>`&lt;underline&gt;`</t>
         </is>
       </c>
       <c r="C46" s="5" t="n"/>
@@ -2283,7 +2279,7 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>`&lt;underline&gt;`</t>
+          <t>`&lt;strikethrough&gt;`</t>
         </is>
       </c>
       <c r="C47" s="5" t="n"/>
@@ -2313,7 +2309,7 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>`&lt;strikethrough&gt;`</t>
+          <t>`&lt;superscript&gt;`</t>
         </is>
       </c>
       <c r="C48" s="5" t="n"/>
@@ -2343,7 +2339,7 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>`&lt;superscript&gt;`</t>
+          <t>`&lt;subscript&gt;`</t>
         </is>
       </c>
       <c r="C49" s="5" t="n"/>
@@ -2373,7 +2369,7 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>`&lt;subscript&gt;`</t>
+          <t>`&lt;handwriting&gt;`</t>
         </is>
       </c>
       <c r="C50" s="5" t="n"/>
@@ -2403,10 +2399,14 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>`&lt;handwriting&gt;`</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="n"/>
+          <t>`&lt;rtl&gt;`</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Indicates right-to-left direction.</t>
+        </is>
+      </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
@@ -2428,32 +2428,32 @@
     <row r="52" ht="17" customHeight="1">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>[05] formatting</t>
+          <t>[06] structural</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>`&lt;rtl&gt;`</t>
+          <t>`&lt;fcel&gt;`</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Indicates right-to-left direction.</t>
+          <t>Indicates the beginning of a full / regular cell.</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Any context that allows raw text content.</t>
+          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
         </is>
       </c>
       <c r="E52" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F52" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G52" s="6" t="b">
-        <v>1</v>
+      <c r="G52" s="1" t="b">
+        <v>0</v>
       </c>
       <c r="H52" s="1" t="b">
         <v>0</v>
@@ -2467,12 +2467,12 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>`&lt;fcel&gt;`</t>
+          <t>`&lt;ecel&gt;`</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a full / regular cell.</t>
+          <t>Indicates the beginning of an empty cell.</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
@@ -2501,12 +2501,12 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ecel&gt;`</t>
+          <t>`&lt;ched&gt;`</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of an empty cell.</t>
+          <t>Indicates the beginning of a column header cell.</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
@@ -2535,12 +2535,12 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ched&gt;`</t>
+          <t>`&lt;rhed&gt;`</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a column header cell.</t>
+          <t>Indicates the beginning of a row header cell.</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
@@ -2561,7 +2561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" ht="17" customHeight="1">
+    <row r="56" ht="34" customHeight="1">
       <c r="A56" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
@@ -2569,12 +2569,12 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>`&lt;rhed&gt;`</t>
+          <t>`&lt;corn&gt;`</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a row header cell.</t>
+          <t>Indicates the beginning of a corner cell, typically the top-left header intersection.</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
@@ -2595,7 +2595,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" ht="34" customHeight="1">
+    <row r="57" ht="17" customHeight="1">
       <c r="A57" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
@@ -2603,12 +2603,12 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>`&lt;corn&gt;`</t>
+          <t>`&lt;srow&gt;`</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a corner cell, typically the top-left header intersection.</t>
+          <t>Indicates the beginning of a section row header.</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
@@ -2629,7 +2629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" ht="17" customHeight="1">
+    <row r="58" ht="51" customHeight="1">
       <c r="A58" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
@@ -2637,12 +2637,12 @@
       </c>
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>`&lt;srow&gt;`</t>
+          <t>`&lt;lcel&gt;`</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a section row header.</t>
+          <t>Left-merge extension token; extends the previous cell horizontally (colspan continuation).</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
@@ -2663,7 +2663,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="51" customHeight="1">
+    <row r="59" ht="34" customHeight="1">
       <c r="A59" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
@@ -2671,12 +2671,12 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>`&lt;lcel&gt;`</t>
+          <t>`&lt;ucel&gt;`</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Left-merge extension token; extends the previous cell horizontally (colspan continuation).</t>
+          <t>Upward-merge extension token; extends the cell above vertically (rowspan continuation)</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
@@ -2697,7 +2697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" ht="34" customHeight="1">
+    <row r="60" ht="51" customHeight="1">
       <c r="A60" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
@@ -2705,12 +2705,12 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ucel&gt;`</t>
+          <t>`&lt;xcel&gt;`</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Upward-merge extension token; extends the cell above vertically (rowspan continuation)</t>
+          <t>Cross/combined span extension token; used where both horizontal and vertical spanning intersect.</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
@@ -2731,7 +2731,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" ht="51" customHeight="1">
+    <row r="61" ht="17" customHeight="1">
       <c r="A61" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
@@ -2739,12 +2739,12 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>`&lt;xcel&gt;`</t>
+          <t>`&lt;nl&gt;`</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Cross/combined span extension token; used where both horizontal and vertical spanning intersect.</t>
+          <t>Denotes the end of a table row.</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
@@ -2765,7 +2765,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" ht="17" customHeight="1">
+    <row r="62" ht="34" customHeight="1">
       <c r="A62" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
@@ -2773,21 +2773,21 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>`&lt;nl&gt;`</t>
+          <t>`&lt;ldiv&gt;`</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Denotes the end of a table row.</t>
+          <t>Indicates the beginning of a list item. It can either be empty or contain a `&lt;marker&gt;`.</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
+          <t>Can only be child of `&lt;list&gt;`.</t>
         </is>
       </c>
       <c r="E62" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F62" s="6" t="b">
         <v>0</v>
@@ -2795,44 +2795,55 @@
       <c r="G62" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="H62" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" ht="34" customHeight="1">
+      <c r="H62" s="1" t="inlineStr">
+        <is>
+          <t>Only `&lt;marker&gt;`</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="17" customHeight="1">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>[06] structural</t>
+          <t>[07] document head</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ldiv&gt;`</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>Indicates the beginning of a list item. It can either be empty or contain a `&lt;marker&gt;`.</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;list&gt;`.</t>
-        </is>
-      </c>
-      <c r="E63" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F63" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G63" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H63" s="1" t="inlineStr">
-        <is>
-          <t>Only `&lt;marker&gt;`</t>
-        </is>
+          <t>`&lt;title&gt;`</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E63" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J63" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="64" ht="17" customHeight="1">
@@ -2843,7 +2854,7 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>`&lt;title&gt;`</t>
+          <t>`&lt;author&gt;`</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -2888,7 +2899,7 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>`&lt;author&gt;`</t>
+          <t>`&lt;date&gt;`</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -2933,41 +2944,30 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>`&lt;date&gt;`</t>
+          <t>`&lt;default_resolution&gt;`</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Defines the default resolution for the document.</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E66" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F66" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G66" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H66" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J66" s="1" t="b">
-        <v>1</v>
+          <t>Can only be child of `&lt;head&gt;`.</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F66" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G66" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H66" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="67" ht="17" customHeight="1">
@@ -2978,30 +2978,41 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>`&lt;default_resolution&gt;`</t>
+          <t>`&lt;page_size&gt;`</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>Defines the default resolution for the document.</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;head&gt;`.</t>
-        </is>
-      </c>
-      <c r="E67" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F67" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G67" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H67" s="6" t="b">
-        <v>0</v>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H67" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J67" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="68" ht="17" customHeight="1">
@@ -3012,7 +3023,7 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>`&lt;page_size&gt;`</t>
+          <t>`&lt;language&gt;`</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -3057,7 +3068,7 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>`&lt;language&gt;`</t>
+          <t>`&lt;generated_by&gt;`</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -3102,7 +3113,7 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>`&lt;generated_by&gt;`</t>
+          <t>`&lt;topic&gt;`</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -3147,7 +3158,7 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>`&lt;topic&gt;`</t>
+          <t>`&lt;summary&gt;`</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -3192,7 +3203,7 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>`&lt;summary&gt;`</t>
+          <t>`&lt;document_hash&gt;`</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -3237,7 +3248,7 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>`&lt;document_hash&gt;`</t>
+          <t>`&lt;licenses&gt;`</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -3282,7 +3293,7 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>`&lt;licenses&gt;`</t>
+          <t>`&lt;data_classification&gt;`</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -3327,7 +3338,7 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>`&lt;data_classification&gt;`</t>
+          <t>`&lt;acceptable_use&gt;`</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -3372,7 +3383,7 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>`&lt;acceptable_use&gt;`</t>
+          <t>`&lt;stewardship&gt;`</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
@@ -3417,7 +3428,7 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>`&lt;stewardship&gt;`</t>
+          <t>`&lt;access_policy&gt;`</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -3462,7 +3473,7 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>`&lt;access_policy&gt;`</t>
+          <t>`&lt;retention_policy&gt;`</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
@@ -3507,7 +3518,7 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>`&lt;retention_policy&gt;`</t>
+          <t>`&lt;compliance_requirements&gt;`</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
@@ -3544,63 +3555,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" ht="17" customHeight="1">
-      <c r="A80" s="7" t="inlineStr">
-        <is>
-          <t>[07] document head</t>
-        </is>
-      </c>
-      <c r="B80" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;compliance_requirements&gt;`</t>
-        </is>
-      </c>
-      <c r="C80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H80" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J80" s="1" t="b">
-        <v>1</v>
-      </c>
+    <row r="80">
+      <c r="A80" s="1" t="n"/>
+      <c r="B80" s="1" t="n"/>
+      <c r="C80" s="1" t="n"/>
+      <c r="D80" s="1" t="n"/>
+      <c r="F80" s="1" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n"/>
-      <c r="B81" s="1" t="n"/>
-      <c r="C81" s="1" t="n"/>
-      <c r="D81" s="1" t="n"/>
-      <c r="F81" s="1" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="4" t="n"/>
+      <c r="A81" s="4" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H80"/>
+  <autoFilter ref="A1:H79"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
@@ -4000,7 +3966,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>{"undefined", "chart", "chemistry"}</t>
+          <t>{"undefined", "chart"}</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">

</xml_diff>

<commit_message>
improve `<location>` handling, various spec refinements (#82)
- Tightened location rules: exactly 4 coords (`x_min,y_min,x_max,y_max`) with normalized order checks and new valid/invalid fixtures.
- Cleaned up `spec.md`: clarified structural constraints, reorganized appendices, and aligned terminology.
- Extended `<marker>` to support element-head metadata (including location) in XSD/Schematron, plus coverage tests.
- Improved DOCX export TOC/heading pagination flow and regenerated reference `.docx`/`.xlsx` outputs.

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -14,7 +14,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'attributes'!$A$1:$E$12</definedName>
   </definedNames>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -610,8 +610,8 @@
     <col width="36.5" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="21"/>
-    <col width="20" customWidth="1" style="1" min="22" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="23"/>
+    <col width="20" customWidth="1" style="1" min="24" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -987,7 +987,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Captures a list. List items are delimited by the respective structural elements. A list item can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
+          <t>Captures a list. List items are started by the respective structural elements (`&lt;ldiv&gt;`). A non-empty `&lt;list&gt;` element body must begin with such a structural element. A list item can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Captures a table in an OTSL-based format. Table cells are delimited by the respective structural elements. A table cell can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
+          <t>Captures a table in an OTSL-based format. Table cells are started by the respective structural elements (`&lt;fcel&gt;` etc). A non-empty `&lt;table&gt;` element body must begin with such a structural element. A table cell can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Captures an index, e.g. for a table of contents or glossary, in an OTSL-based format. Cells are delimited by the respective structural elements. A cell can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
+          <t>Captures an index, e.g. for a table of contents or glossary, in an OTSL-based format. Index cells are started by the respective structural elements (`&lt;fcel&gt;` etc). A non-empty `&lt;index&gt;` element body must begin with such a structural element. A cell can be defined without a wrapping tag, i.e. as pure (optional) element head followed by raw text; this is called an "virtual `&lt;text&gt;`" and is handled exactly like a regular `&lt;text&gt;` element.</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Can contain a `&lt;src&gt;` for image bytes or reference. Additionally, the element body may begin with a `&lt;table&gt;` in case of `&lt;picture class="chart"&gt;`.</t>
+          <t>Element body can generally only contain a `&lt;src&gt;`, for image bytes or reference. Additionally, in case of `&lt;picture class="chart"&gt;` (and only then) the element body may contain a `&lt;table&gt;`, in which case it must begin with it.</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -1197,8 +1197,10 @@
       <c r="G16" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="H16" s="1" t="b">
-        <v>1</v>
+      <c r="H16" s="1" t="inlineStr">
+        <is>
+          <t>Not allowed (except `&lt;table&gt;` in case of `&lt;picture class="chart"&gt;`)</t>
+        </is>
       </c>
       <c r="I16" s="1" t="b">
         <v>1</v>
@@ -1694,7 +1696,7 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Used to store additional or derived information regarding the respective component.</t>
+          <t>Optional part of the element head; used to store additional or derived information regarding the respective component.</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -1734,7 +1736,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Custom metadata, e.g. for application-specific purposes.</t>
+          <t>Optional part of the element head; custom metadata, e.g. for application-specific purposes.</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -1771,7 +1773,7 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Coordinate system is the bottom-left corner of the page.</t>
+          <t>Optional part of the element head; coordinate system is the top-left corner of the page. When present, appears in sequence of 4 `&lt;location&gt;` instances, representing x0, y0, x1, y1. The following must then hold: `x0_norm&lt;=x1_norm` and `y0_norm&lt;=y1_norm`(i.e. first top-left point then bottom-right point), whereby `*_norm` is the respective coordinate normalized to its effective resolution.</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -3771,6 +3773,11 @@
           <t>Integer within [0, `location.resolution`)</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Coordinate w.r.t. top-left corner.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4047,7 +4054,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>A string that identifies a thread.</t>
+          <t>The ID of the thread. All `&lt;thread&gt;` elements that share a given `thread_id` must be under the same host element type (e.g. all under `&lt;text&gt;`, not mixed `&lt;text&gt;` and `&lt;picture&gt;`).</t>
         </is>
       </c>
     </row>
@@ -4096,7 +4103,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>The ID of the referenced thread.</t>
+          <t>The ID of the referenced thread. This must be defined by at least one `&lt;thread&gt;` in the document.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
enforce field scope rules, expand recommendation guidance (#83)
- Add Schematron rules to enforce field placement (`field_heading`/`field_item` under `field_region`, `key`/`value` under `field_item`) and own-key cardinality per `field_item`.
- Update valid/invalid XML fixtures to cover misplaced elements, duplicate own keys, and nested `field_item` key scoping.
- Refine spec language by renaming Appendix B to broader recommendations and documenting custom vocabulary naming/namespacing guidance.

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -14,7 +14,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'attributes'!$A$1:$E$12</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -610,8 +610,8 @@
     <col width="36.5" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="23"/>
-    <col width="20" customWidth="1" style="1" min="24" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="25"/>
+    <col width="20" customWidth="1" style="1" min="26" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1674,7 +1674,7 @@
         <v>0</v>
       </c>
       <c r="G29" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H29" s="1" t="b">
         <v>0</v>
@@ -1736,7 +1736,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Optional part of the element head; custom metadata, e.g. for application-specific purposes.</t>
+          <t>Optional part of the element head; custom metadata, e.g. for application-specific purposes. See [Appendix B: Recommendations](#appendix-b-recommendations) for naming and namespacing guidance for custom vocabularies.</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">

</xml_diff>

<commit_message>
prepare release v0.4.0 (#86)
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -3657,12 +3657,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Optional; default: "0.3"</t>
+          <t>Optional; default: "0.4"</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>{"0.3"}</t>
+          <t>{"0.4"}</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">

</xml_diff>

<commit_message>
add `<layer>`, document tokenization guidelines (#87)
- Add optional `<layer>` to the element head (spec & validator).
- Add token vocabulary guidance.

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="1" state="visible" r:id="rId1"/>
@@ -610,8 +610,8 @@
     <col width="36.5" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="25"/>
-    <col width="20" customWidth="1" style="1" min="26" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="29"/>
+    <col width="20" customWidth="1" style="1" min="30" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1544,8 +1544,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Optional part of the element head; serves for establishing a logical document component. This can be useful for capturing fragmented components, e.g. spanning multiple bounding boxes (e.g. cross-column) or pages, or for defining anchors for cross references.&lt;br/&gt;
-To capture a fragmented component, we define separate instances of the respective element and use a `&lt;thread&gt;` with the same `thread_id` attribute for all of them</t>
+          <t>Optional part of the element head; serves for establishing a logical document component. This can be useful for capturing fragmented components, e.g. spanning multiple bounding boxes (e.g. cross-column) or pages, or for defining anchors for cross references. To capture a fragmented component, we define separate instances of the respective element and use a `&lt;thread&gt;` with the same `thread_id` attribute for all of them</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -1848,7 +1847,11 @@
           <t>`&lt;layer&gt;`</t>
         </is>
       </c>
-      <c r="C34" s="5" t="n"/>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>The conceptual layer of the host element in the document.</t>
+        </is>
+      </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
           <t>Can only be child of a semantic element.</t>
@@ -1867,9 +1870,6 @@
         <v>0</v>
       </c>
       <c r="I34" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J34" s="1" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3875,7 +3875,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>`class`</t>
+          <t>`value`</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -3885,7 +3885,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>{"body", "furniture", "background", "invisible", "notes"}</t>
+          <t>{"body", "background", "furniture"}</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>The layer value: "body" is for the document's main content, "background" is for watermarks and other background components, while "furniture" is the fallback for any supplementary components not contributing to the document's main content, such as navigation or decorations.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prepare release v0.5.0 (#89)
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -3657,12 +3657,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Optional; default: "0.4"</t>
+          <t>Optional; default: "0.5"</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>{"0.4"}</t>
+          <t>{"0.5"}</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">

</xml_diff>

<commit_message>
allow full sem. body in `<picture>`, add `<tabular>` for chart tables (#90)
- Allow a full semantic body in `<picture>` (text, nested pictures, etc.) via XSD and Schematron updates
- Introduce `<tabular>` as the OTSL payload for `<picture class="chart">`, with `src` first and `tabular` immediately after when both are present
- Refresh `form-examples.md` from legacy `form`/`form_item`/`form_heading` to `field_region`/`field_item`/`field_heading`
- Add markdown XML-snippet validation (`utils/validate_markdown_snippets.py`, `tests/test_markdown_snippets.py`)
- Regenerate spec reference exports and fix the README CONTRIBUTING link

Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="66640" yWindow="4520" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="1" state="visible" r:id="rId1"/>
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="attributes" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'elements'!$A$1:$H$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'attributes'!$A$1:$E$12</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -38,6 +38,19 @@
     <font>
       <name val="Aptos Narrow"/>
       <color theme="1"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <color rgb="FF000000"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
@@ -62,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -87,6 +100,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -601,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J81"/>
+  <dimension ref="A1:J82"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20" defaultRowHeight="16"/>
   <cols>
     <col width="27.1640625" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -610,8 +629,8 @@
     <col width="36.5" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="17.5" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
     <col width="17.1640625" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="20" customWidth="1" style="1" min="7" max="29"/>
-    <col width="20" customWidth="1" style="1" min="30" max="16384"/>
+    <col width="20" customWidth="1" style="1" min="7" max="31"/>
+    <col width="20" customWidth="1" style="1" min="32" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -816,7 +835,11 @@
           <t>`&lt;heading&gt;`</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n"/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Captures a document heading.</t>
+        </is>
+      </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Any context that allows semantic elements.</t>
@@ -849,7 +872,11 @@
           <t>`&lt;footnote&gt;`</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n"/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Captures footnote content.</t>
+        </is>
+      </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Any context that allows semantic elements.</t>
@@ -882,7 +909,11 @@
           <t>`&lt;page_header&gt;`</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n"/>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Captures page header content (material repeated at the top of a page).</t>
+        </is>
+      </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Any context that allows semantic elements.</t>
@@ -915,7 +946,11 @@
           <t>`&lt;page_footer&gt;`</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n"/>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Captures page footer content (material repeated at the bottom of a page).</t>
+        </is>
+      </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Any context that allows semantic elements.</t>
@@ -1033,7 +1068,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Any context that allows semantic elements. And additionally as the first element of the element body of `&lt;picture class="chart"&gt;`.</t>
+          <t>Any context that allows semantic elements.</t>
         </is>
       </c>
       <c r="E12" s="6" t="b">
@@ -1145,7 +1180,11 @@
           <t>`&lt;code&gt;`</t>
         </is>
       </c>
-      <c r="C15" s="5" t="n"/>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Captures a code snippet, either as a standalone block or inlined within a semantic element. For language classification, use a `&lt;label&gt;`in the element head (see [Appendix B: Recommendations](#appendix-b-recommendations)).</t>
+        </is>
+      </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Any context that allows semantic elements.</t>
@@ -1180,7 +1219,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Element body can generally only contain a `&lt;src&gt;`, for image bytes or reference. Additionally, in case of `&lt;picture class="chart"&gt;` (and only then) the element body may contain a `&lt;table&gt;`, in which case it must begin with it.</t>
+          <t>The element body begins with a picture-specific sequence, followed by content allowed in any other semantic element body. The picture-specific sequence is:&lt;ul&gt;&lt;li&gt;an optional `&lt;src&gt;` element&lt;/li&gt;&lt;li&gt;an optional `&lt;tabular&gt;` element (only allowed for `&lt;picture class="chart"&gt;`)&lt;/li&gt;&lt;/ul&gt;</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -1197,10 +1236,8 @@
       <c r="G16" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="H16" s="1" t="inlineStr">
-        <is>
-          <t>Not allowed (except `&lt;table&gt;` in case of `&lt;picture class="chart"&gt;`)</t>
-        </is>
+      <c r="H16" s="1" t="b">
+        <v>1</v>
       </c>
       <c r="I16" s="1" t="b">
         <v>1</v>
@@ -1217,7 +1254,11 @@
           <t>`&lt;marker&gt;`</t>
         </is>
       </c>
-      <c r="C17" s="5" t="n"/>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Captures the visible glyph or identifier (e.g. number) of a marker, e.g. in the context of a list item.</t>
+        </is>
+      </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Any context that allows semantic elements.</t>
@@ -1287,7 +1328,11 @@
           <t>`&lt;field_heading&gt;`</t>
         </is>
       </c>
-      <c r="C19" s="5" t="n"/>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Field heading within a `&lt;field_region&gt;; analogous to `&lt;heading&gt;` but scoped to field structures.</t>
+        </is>
+      </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
           <t>Can only be descendant of `&lt;field_region&gt;`.</t>
@@ -1475,7 +1520,7 @@
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Can only be part of the element head of a semantic element.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E24" s="6" t="b">
@@ -1512,7 +1557,7 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E25" s="6" t="b">
@@ -1549,7 +1594,7 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E26" s="6" t="b">
@@ -1586,7 +1631,7 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E27" s="6" t="b">
@@ -1626,7 +1671,7 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element. Mutually exclusive with `&lt;href&gt;`.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E28" s="6" t="b">
@@ -1663,7 +1708,7 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element. Mutually exclusive with `&lt;xref&gt;`.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E29" s="6" t="b">
@@ -1700,7 +1745,7 @@
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E30" s="6" t="b">
@@ -1740,7 +1785,7 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E31" s="6" t="b">
@@ -1777,7 +1822,7 @@
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E32" s="6" t="b">
@@ -1814,7 +1859,7 @@
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E33" s="6" t="b">
@@ -1854,7 +1899,7 @@
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of a semantic element.</t>
+          <t>Can only be part of the [element head](#element-head) of a semantic element.</t>
         </is>
       </c>
       <c r="E34" s="6" t="b">
@@ -2107,7 +2152,7 @@
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;picture&gt;`.</t>
+          <t>Can only be part of the picture-specific element body sequence of `&lt;picture&gt;`.</t>
         </is>
       </c>
       <c r="E41" s="6" t="b">
@@ -2123,7 +2168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" ht="17" customHeight="1">
+    <row r="42" ht="51" customHeight="1">
       <c r="A42" s="7" t="inlineStr">
         <is>
           <t>[04] payload</t>
@@ -2131,27 +2176,36 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>`&lt;checkbox&gt;`</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="n"/>
+          <t>`&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Structured tabular data. Uses the same cell model as `&lt;table&gt;`, but without an element head of its own.</t>
+        </is>
+      </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Any context that allows raw text content.</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F42" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G42" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H42" s="1" t="b">
-        <v>0</v>
-      </c>
+          <t>Can only be part of the picture-specific element body sequence of [`&lt;picture class="chart"&gt;`](#picture).</t>
+        </is>
+      </c>
+      <c r="E42" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
+          <t>Only on cell level, in case of virtual `&lt;text&gt;`</t>
+        </is>
+      </c>
+      <c r="G42" s="10" t="inlineStr">
+        <is>
+          <t>Only on cell level, in case of virtual `&lt;text&gt;`</t>
+        </is>
+      </c>
+      <c r="H42" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I42" s="10" t="n"/>
     </row>
     <row r="43" ht="17" customHeight="1">
       <c r="A43" s="7" t="inlineStr">
@@ -2161,23 +2215,27 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>`&lt;content&gt;`</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="n"/>
+          <t>`&lt;checkbox&gt;`</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Empty element representing checkbox selection state.</t>
+        </is>
+      </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
         </is>
       </c>
       <c r="E43" s="6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F43" s="6" t="b">
         <v>0</v>
       </c>
       <c r="G43" s="1" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H43" s="1" t="b">
         <v>0</v>
@@ -2186,15 +2244,19 @@
     <row r="44" ht="17" customHeight="1">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>[05] formatting</t>
+          <t>[04] payload</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>`&lt;bold&gt;`</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="n"/>
+          <t>`&lt;content&gt;`</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Whitespace-preserving text container. Retains all whitespace within the element (equivalent to `xml:space="preserve"`), enabling use in whitespace-sensitive scenarios such as code blocks. XML special characters may alternatively be conveyed via CDATA.</t>
+        </is>
+      </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
@@ -2206,7 +2268,7 @@
       <c r="F44" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G44" s="6" t="b">
+      <c r="G44" s="1" t="b">
         <v>1</v>
       </c>
       <c r="H44" s="1" t="b">
@@ -2221,10 +2283,14 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>`&lt;italic&gt;`</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="n"/>
+          <t>`&lt;bold&gt;`</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Indicates bold formatting.</t>
+        </is>
+      </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
@@ -2251,10 +2317,14 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>`&lt;underline&gt;`</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="n"/>
+          <t>`&lt;italic&gt;`</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Indicates italic formatting.</t>
+        </is>
+      </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
@@ -2281,10 +2351,14 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>`&lt;strikethrough&gt;`</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="n"/>
+          <t>`&lt;underline&gt;`</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Indicates underlined formatting.</t>
+        </is>
+      </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
@@ -2311,10 +2385,14 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>`&lt;superscript&gt;`</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="n"/>
+          <t>`&lt;strikethrough&gt;`</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Indicates struck-through formatting.</t>
+        </is>
+      </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
@@ -2341,10 +2419,14 @@
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>`&lt;subscript&gt;`</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="n"/>
+          <t>`&lt;superscript&gt;`</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Indicates superscript formatting.</t>
+        </is>
+      </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
@@ -2371,10 +2453,14 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>`&lt;handwriting&gt;`</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="n"/>
+          <t>`&lt;subscript&gt;`</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Indicates subscript formatting.</t>
+        </is>
+      </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
           <t>Any context that allows raw text content.</t>
@@ -2401,12 +2487,12 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>`&lt;rtl&gt;`</t>
+          <t>`&lt;handwriting&gt;`</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Indicates right-to-left direction.</t>
+          <t>Indicates handwritten text.</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
@@ -2430,32 +2516,32 @@
     <row r="52" ht="17" customHeight="1">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>[06] structural</t>
+          <t>[05] formatting</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>`&lt;fcel&gt;`</t>
+          <t>`&lt;rtl&gt;`</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a full / regular cell.</t>
+          <t>Indicates right-to-left direction.</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
+          <t>Any context that allows raw text content.</t>
         </is>
       </c>
       <c r="E52" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F52" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G52" s="1" t="b">
-        <v>0</v>
+      <c r="G52" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="H52" s="1" t="b">
         <v>0</v>
@@ -2469,17 +2555,17 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ecel&gt;`</t>
+          <t>`&lt;fcel&gt;`</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of an empty cell.</t>
+          <t>Indicates the beginning of a full / regular cell.</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
         </is>
       </c>
       <c r="E53" s="6" t="b">
@@ -2503,17 +2589,17 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>`&lt;ched&gt;`</t>
+          <t>`&lt;ecel&gt;`</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Indicates the beginning of a column header cell.</t>
+          <t>Indicates the beginning of an empty cell.</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
         </is>
       </c>
       <c r="E54" s="6" t="b">
@@ -2537,315 +2623,304 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
+          <t>`&lt;ched&gt;`</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Indicates the beginning of a column header cell.</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F55" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G55" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H55" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" ht="17" customHeight="1">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>[06] structural</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
           <t>`&lt;rhed&gt;`</t>
         </is>
       </c>
-      <c r="C55" s="5" t="inlineStr">
+      <c r="C56" s="5" t="inlineStr">
         <is>
           <t>Indicates the beginning of a row header cell.</t>
         </is>
       </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
-        </is>
-      </c>
-      <c r="E55" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F55" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G55" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H55" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" ht="34" customHeight="1">
-      <c r="A56" s="7" t="inlineStr">
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F56" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G56" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H56" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" ht="34" customHeight="1">
+      <c r="A57" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B56" s="5" t="inlineStr">
+      <c r="B57" s="5" t="inlineStr">
         <is>
           <t>`&lt;corn&gt;`</t>
         </is>
       </c>
-      <c r="C56" s="5" t="inlineStr">
+      <c r="C57" s="5" t="inlineStr">
         <is>
           <t>Indicates the beginning of a corner cell, typically the top-left header intersection.</t>
         </is>
       </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F56" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G56" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H56" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" ht="17" customHeight="1">
-      <c r="A57" s="7" t="inlineStr">
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F57" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G57" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H57" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" ht="17" customHeight="1">
+      <c r="A58" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B57" s="5" t="inlineStr">
+      <c r="B58" s="5" t="inlineStr">
         <is>
           <t>`&lt;srow&gt;`</t>
         </is>
       </c>
-      <c r="C57" s="5" t="inlineStr">
+      <c r="C58" s="5" t="inlineStr">
         <is>
           <t>Indicates the beginning of a section row header.</t>
         </is>
       </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
-        </is>
-      </c>
-      <c r="E57" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F57" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G57" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H57" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" ht="51" customHeight="1">
-      <c r="A58" s="7" t="inlineStr">
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F58" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G58" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H58" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" ht="51" customHeight="1">
+      <c r="A59" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B58" s="5" t="inlineStr">
+      <c r="B59" s="5" t="inlineStr">
         <is>
           <t>`&lt;lcel&gt;`</t>
         </is>
       </c>
-      <c r="C58" s="5" t="inlineStr">
+      <c r="C59" s="5" t="inlineStr">
         <is>
           <t>Left-merge extension token; extends the previous cell horizontally (colspan continuation).</t>
         </is>
       </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F58" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G58" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H58" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" ht="34" customHeight="1">
-      <c r="A59" s="7" t="inlineStr">
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F59" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G59" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H59" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" ht="34" customHeight="1">
+      <c r="A60" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B59" s="5" t="inlineStr">
+      <c r="B60" s="5" t="inlineStr">
         <is>
           <t>`&lt;ucel&gt;`</t>
         </is>
       </c>
-      <c r="C59" s="5" t="inlineStr">
+      <c r="C60" s="5" t="inlineStr">
         <is>
           <t>Upward-merge extension token; extends the cell above vertically (rowspan continuation)</t>
         </is>
       </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
-        </is>
-      </c>
-      <c r="E59" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F59" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G59" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H59" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" ht="51" customHeight="1">
-      <c r="A60" s="7" t="inlineStr">
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F60" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G60" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H60" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" ht="51" customHeight="1">
+      <c r="A61" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B60" s="5" t="inlineStr">
+      <c r="B61" s="5" t="inlineStr">
         <is>
           <t>`&lt;xcel&gt;`</t>
         </is>
       </c>
-      <c r="C60" s="5" t="inlineStr">
+      <c r="C61" s="5" t="inlineStr">
         <is>
           <t>Cross/combined span extension token; used where both horizontal and vertical spanning intersect.</t>
         </is>
       </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
-        </is>
-      </c>
-      <c r="E60" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F60" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G60" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H60" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" ht="17" customHeight="1">
-      <c r="A61" s="7" t="inlineStr">
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F61" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G61" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H61" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" ht="17" customHeight="1">
+      <c r="A62" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B61" s="5" t="inlineStr">
+      <c r="B62" s="5" t="inlineStr">
         <is>
           <t>`&lt;nl&gt;`</t>
         </is>
       </c>
-      <c r="C61" s="5" t="inlineStr">
+      <c r="C62" s="5" t="inlineStr">
         <is>
           <t>Denotes the end of a table row.</t>
         </is>
       </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>Can only be child of `&lt;table&gt;` or `&lt;index&gt;`</t>
-        </is>
-      </c>
-      <c r="E61" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F61" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G61" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H61" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" ht="34" customHeight="1">
-      <c r="A62" s="7" t="inlineStr">
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Can only be child of `&lt;table&gt;`, `&lt;index&gt;`, or `&lt;tabular&gt;`</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F62" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G62" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H62" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" ht="34" customHeight="1">
+      <c r="A63" s="7" t="inlineStr">
         <is>
           <t>[06] structural</t>
         </is>
       </c>
-      <c r="B62" s="5" t="inlineStr">
+      <c r="B63" s="5" t="inlineStr">
         <is>
           <t>`&lt;ldiv&gt;`</t>
         </is>
       </c>
-      <c r="C62" s="5" t="inlineStr">
+      <c r="C63" s="5" t="inlineStr">
         <is>
           <t>Indicates the beginning of a list item. It can either be empty or contain a `&lt;marker&gt;`.</t>
         </is>
       </c>
-      <c r="D62" s="5" t="inlineStr">
+      <c r="D63" s="5" t="inlineStr">
         <is>
           <t>Can only be child of `&lt;list&gt;`.</t>
         </is>
       </c>
-      <c r="E62" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F62" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G62" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H62" s="1" t="inlineStr">
+      <c r="E63" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F63" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G63" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="H63" s="1" t="inlineStr">
         <is>
           <t>Only `&lt;marker&gt;`</t>
         </is>
-      </c>
-    </row>
-    <row r="63" ht="17" customHeight="1">
-      <c r="A63" s="7" t="inlineStr">
-        <is>
-          <t>[07] document head</t>
-        </is>
-      </c>
-      <c r="B63" s="5" t="inlineStr">
-        <is>
-          <t>`&lt;title&gt;`</t>
-        </is>
-      </c>
-      <c r="C63" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D63" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E63" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F63" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G63" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H63" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J63" s="1" t="b">
-        <v>1</v>
       </c>
     </row>
     <row r="64" ht="17" customHeight="1">
@@ -2856,7 +2931,7 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>`&lt;author&gt;`</t>
+          <t>`&lt;title&gt;`</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -2901,7 +2976,7 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>`&lt;date&gt;`</t>
+          <t>`&lt;author&gt;`</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -2946,30 +3021,41 @@
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>`&lt;default_resolution&gt;`</t>
+          <t>`&lt;date&gt;`</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Defines the default resolution for the document.</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>Can only be child of `&lt;head&gt;`.</t>
-        </is>
-      </c>
-      <c r="E66" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="F66" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G66" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H66" s="6" t="b">
-        <v>0</v>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F66" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G66" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J66" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="67" ht="17" customHeight="1">
@@ -2980,41 +3066,30 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>`&lt;page_size&gt;`</t>
+          <t>`&lt;default_resolution&gt;`</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Defines the default resolution for the document.</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E67" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F67" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G67" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H67" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J67" s="1" t="b">
-        <v>1</v>
+          <t>Can only be child of `&lt;head&gt;`.</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F67" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G67" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H67" s="6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="68" ht="17" customHeight="1">
@@ -3025,7 +3100,7 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>`&lt;language&gt;`</t>
+          <t>`&lt;page_size&gt;`</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -3070,7 +3145,7 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>`&lt;generated_by&gt;`</t>
+          <t>`&lt;language&gt;`</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -3115,7 +3190,7 @@
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>`&lt;topic&gt;`</t>
+          <t>`&lt;generated_by&gt;`</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -3160,7 +3235,7 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>`&lt;summary&gt;`</t>
+          <t>`&lt;topic&gt;`</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -3205,7 +3280,7 @@
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>`&lt;document_hash&gt;`</t>
+          <t>`&lt;summary&gt;`</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -3250,7 +3325,7 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>`&lt;licenses&gt;`</t>
+          <t>`&lt;document_hash&gt;`</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -3295,7 +3370,7 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>`&lt;data_classification&gt;`</t>
+          <t>`&lt;licenses&gt;`</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -3340,7 +3415,7 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>`&lt;acceptable_use&gt;`</t>
+          <t>`&lt;data_classification&gt;`</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -3385,7 +3460,7 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>`&lt;stewardship&gt;`</t>
+          <t>`&lt;acceptable_use&gt;`</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
@@ -3430,7 +3505,7 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>`&lt;access_policy&gt;`</t>
+          <t>`&lt;stewardship&gt;`</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -3475,7 +3550,7 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>`&lt;retention_policy&gt;`</t>
+          <t>`&lt;access_policy&gt;`</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
@@ -3520,55 +3595,100 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
+          <t>`&lt;retention_policy&gt;`</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F79" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G79" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H79" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J79" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" ht="17" customHeight="1">
+      <c r="A80" s="7" t="inlineStr">
+        <is>
+          <t>[07] document head</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
           <t>`&lt;compliance_requirements&gt;`</t>
         </is>
       </c>
-      <c r="C79" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="D79" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="E79" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="F79" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G79" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="H79" s="6" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="J79" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="1" t="n"/>
-      <c r="B80" s="1" t="n"/>
-      <c r="C80" s="1" t="n"/>
-      <c r="D80" s="1" t="n"/>
-      <c r="F80" s="1" t="n"/>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J80" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="81">
-      <c r="A81" s="4" t="n"/>
+      <c r="A81" s="1" t="n"/>
+      <c r="B81" s="1" t="n"/>
+      <c r="C81" s="1" t="n"/>
+      <c r="D81" s="1" t="n"/>
+      <c r="F81" s="1" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H79"/>
+  <autoFilter ref="A1:H80"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
@@ -3770,7 +3890,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Integer within [0, `location.resolution`)</t>
+          <t>Integer within [0, `location@resolution`)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -3915,6 +4035,11 @@
           <t>Positive integer</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>The heading depth (1 = top-level).</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3937,6 +4062,11 @@
           <t>{"read_only", "fillable"}</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>The value type.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3959,6 +4089,11 @@
           <t>{"unordered", "ordered"}</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>The list type.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4008,6 +4143,11 @@
           <t>{"unselected", "selected"}</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>The checkbox type.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4185,6 +4325,11 @@
       <c r="D24" t="inlineStr">
         <is>
           <t>Positive integer</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>The field heading depth (1 = top-level).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
prepare release v0.6.0 (#92)
Signed-off-by: Panos Vagenas <pva@zurich.ibm.com>
</commit_message>
<xml_diff>
--- a/reference/input/reference.xlsx
+++ b/reference/input/reference.xlsx
@@ -3777,12 +3777,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Optional; default: "0.5"</t>
+          <t>Optional; default: "0.6"</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>{"0.5"}</t>
+          <t>{"0.6"}</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">

</xml_diff>